<commit_message>
feat(exe): add single EXE builder with GUI interface
- Add build_single_exe.py for creating single executable file
- Create graphical user interface with tkinter
- Include all dependencies and EdgeDriver in single EXE
- Add PyInstaller configuration for Windows builds
- Implement GUI features: PO input, CSV import, progress tracking
- Add settings: headless mode, max POs limit
- Include sample data and validation
- Create comprehensive README for single EXE version
- Update main README to focus on single EXE as recommended option
- Remove alternative portable package options

Single EXE features:
- Zero installation required
- Graphical user interface
- All dependencies embedded
- Stable EdgeDriver included
- Portable to any Windows machine
- User-friendly PO input and validation
- Progress tracking and error handling
</commit_message>
<xml_diff>
--- a/data/input/input.xlsx
+++ b/data/input/input.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,12 +50,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="0090EE90"/>
         <bgColor rgb="0090EE90"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFB6C1"/>
-        <bgColor rgb="00FFB6C1"/>
       </patternFill>
     </fill>
     <fill>
@@ -83,14 +77,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,9 +544,9 @@
           <t>PO16400507</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -565,11 +558,11 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025-08-04 23:04:41</t>
+          <t>2025-08-04 23:38:49</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -604,7 +597,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-08-04 23:04:41</t>
+          <t>2025-08-04 23:38:50</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -621,9 +614,9 @@
           <t>PO15377448</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -635,11 +628,11 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2025-08-04 23:04:53</t>
+          <t>2025-08-04 23:39:01</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -894,9 +887,9 @@
           <t>PO15682304</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -908,11 +901,11 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-08-04 23:05:06</t>
+          <t>2025-08-04 23:39:12</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -972,9 +965,9 @@
           <t>PO14174358</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -986,11 +979,11 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-08-04 23:05:18</t>
+          <t>2025-08-04 23:39:23</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1167,22 +1160,38 @@
           <t>PO16521185</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DELIVERECT-0050576836</t>
+        </is>
+      </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:39:32</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>DELIVERECT-0050576836/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16521185</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1190,22 +1199,38 @@
           <t>PO16546302</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312</t>
+        </is>
+      </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:39:39</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16546302</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1213,22 +1238,38 @@
           <t>PO16505408</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Gartner_UK_Ltd-0000920176</t>
+        </is>
+      </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:39:48</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Gartner_UK_Ltd-0000920176/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16505408</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1236,9 +1277,9 @@
           <t>PO16576174</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>NO_ATTACHMENTS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1248,10 +1289,18 @@
       <c r="E22" t="n">
         <v>0</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:39:49</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16576174</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1259,22 +1308,38 @@
           <t>PO15345517</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AVANADE_UK_LIMITED-0009842181</t>
+        </is>
+      </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:40:03</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>AVANADE_UK_LIMITED-0009842181/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15345517</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1282,22 +1347,38 @@
           <t>PO16393497</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>NEEM_CONSULTING_LIMITED-0001080021</t>
+        </is>
+      </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:40:14</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NEEM_CONSULTING_LIMITED-0001080021/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16393497</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1305,22 +1386,38 @@
           <t>PO16330706</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DELOITTE_TOUCHE_TOHMATSU_INDIA_LLP-0050532353</t>
+        </is>
+      </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:40:22</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>DELOITTE_TOUCHE_TOHMATSU_INDIA_LLP-0050532353/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16330706</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1328,7 +1425,7 @@
           <t>PO16370617</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1351,7 +1448,7 @@
           <t>PO15776178</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1374,7 +1471,7 @@
           <t>PO16110682</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1397,7 +1494,7 @@
           <t>PO16295766</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1420,7 +1517,7 @@
           <t>PO16263753</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1443,7 +1540,7 @@
           <t>PO16243786</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1466,7 +1563,7 @@
           <t>PO15190568</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1489,7 +1586,7 @@
           <t>PO15279299</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1512,7 +1609,7 @@
           <t>PO16311692</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1535,7 +1632,7 @@
           <t>PO16508611</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1558,7 +1655,7 @@
           <t>PO16291902</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1581,7 +1678,7 @@
           <t>PO16291905</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1604,7 +1701,7 @@
           <t>PO16362026</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1627,7 +1724,7 @@
           <t>PO16401398</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1650,7 +1747,7 @@
           <t>PO16258825</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1673,7 +1770,7 @@
           <t>PO16329900</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1696,7 +1793,7 @@
           <t>PO16307414</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1719,7 +1816,7 @@
           <t>PO15910712</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1742,7 +1839,7 @@
           <t>PO16323977</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1765,7 +1862,7 @@
           <t>PO16400408</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1788,7 +1885,7 @@
           <t>PO16359621</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1811,7 +1908,7 @@
           <t>PO16242475</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1834,7 +1931,7 @@
           <t>PO15436910</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1857,7 +1954,7 @@
           <t>PO15179449</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1880,7 +1977,7 @@
           <t>PO15837036</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1903,7 +2000,7 @@
           <t>PO16478674</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1926,7 +2023,7 @@
           <t>PO16408165</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1949,7 +2046,7 @@
           <t>PO15285807</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1972,7 +2069,7 @@
           <t>PO16447367</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -1995,7 +2092,7 @@
           <t>PO16456067</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2018,7 +2115,7 @@
           <t>PO16493712</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2041,7 +2138,7 @@
           <t>PO16407260</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2064,7 +2161,7 @@
           <t>PO16353483</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2087,7 +2184,7 @@
           <t>PO15287725</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2110,7 +2207,7 @@
           <t>PO16413103</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2133,7 +2230,7 @@
           <t>PO16465704</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2156,7 +2253,7 @@
           <t>PO16510823</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2179,7 +2276,7 @@
           <t>PO16224968</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2202,7 +2299,7 @@
           <t>PO16556376</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2225,7 +2322,7 @@
           <t>PO16488279</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2248,7 +2345,7 @@
           <t>PO15630093</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2271,7 +2368,7 @@
           <t>PO16262209</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2294,7 +2391,7 @@
           <t>PO16477243</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2317,7 +2414,7 @@
           <t>PO15617175</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2340,7 +2437,7 @@
           <t>PO16384342</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2363,7 +2460,7 @@
           <t>PO15285778</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2386,7 +2483,7 @@
           <t>PO16398622</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2409,7 +2506,7 @@
           <t>PO15154338</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2432,7 +2529,7 @@
           <t>PO16207336</t>
         </is>
       </c>
-      <c r="B74" s="4" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2455,7 +2552,7 @@
           <t>PO16269922</t>
         </is>
       </c>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2478,7 +2575,7 @@
           <t>PO16400435</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2501,7 +2598,7 @@
           <t>PO16264501</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2524,7 +2621,7 @@
           <t>PO14729307</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2547,7 +2644,7 @@
           <t>PO16105473</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2570,7 +2667,7 @@
           <t>PO15437050</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2593,7 +2690,7 @@
           <t>PO15617177</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2616,7 +2713,7 @@
           <t>PO16497039</t>
         </is>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2639,7 +2736,7 @@
           <t>PO16400407</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2662,7 +2759,7 @@
           <t>PO16219761</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2685,7 +2782,7 @@
           <t>PO15694773</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2708,7 +2805,7 @@
           <t>PO16539229</t>
         </is>
       </c>
-      <c r="B86" s="4" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2731,7 +2828,7 @@
           <t>PO16233980</t>
         </is>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2754,7 +2851,7 @@
           <t>PO13068435</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2777,7 +2874,7 @@
           <t>PO16366575</t>
         </is>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2800,7 +2897,7 @@
           <t>PO16343173</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2823,7 +2920,7 @@
           <t>PO16253759</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2846,7 +2943,7 @@
           <t>PO15285775</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B92" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2869,7 +2966,7 @@
           <t>PO16240302</t>
         </is>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B93" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2892,7 +2989,7 @@
           <t>PO14752945</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B94" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2915,7 +3012,7 @@
           <t>PO16393498</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B95" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2938,7 +3035,7 @@
           <t>PO13081743</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2961,7 +3058,7 @@
           <t>PO15617218</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B97" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2984,7 +3081,7 @@
           <t>PO15285806</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3007,7 +3104,7 @@
           <t>PO16253702</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3030,7 +3127,7 @@
           <t>PO16330407</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3053,7 +3150,7 @@
           <t>PO16322561</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B101" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3076,7 +3173,7 @@
           <t>PO13019654</t>
         </is>
       </c>
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3099,7 +3196,7 @@
           <t>PO16188865</t>
         </is>
       </c>
-      <c r="B103" s="4" t="inlineStr">
+      <c r="B103" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3122,7 +3219,7 @@
           <t>PO15715793</t>
         </is>
       </c>
-      <c r="B104" s="4" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3145,7 +3242,7 @@
           <t>PO16380788</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="B105" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3168,7 +3265,7 @@
           <t>PO16258716</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B106" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3191,7 +3288,7 @@
           <t>PO16191725</t>
         </is>
       </c>
-      <c r="B107" s="4" t="inlineStr">
+      <c r="B107" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3214,7 +3311,7 @@
           <t>PO15718023</t>
         </is>
       </c>
-      <c r="B108" s="4" t="inlineStr">
+      <c r="B108" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3237,7 +3334,7 @@
           <t>PO16258379</t>
         </is>
       </c>
-      <c r="B109" s="4" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3260,7 +3357,7 @@
           <t>PO14769933</t>
         </is>
       </c>
-      <c r="B110" s="4" t="inlineStr">
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3283,7 +3380,7 @@
           <t>PO15980633</t>
         </is>
       </c>
-      <c r="B111" s="4" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3306,7 +3403,7 @@
           <t>PO16383021</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3329,7 +3426,7 @@
           <t>PO14769930</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B113" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3352,7 +3449,7 @@
           <t>PO16042562</t>
         </is>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B114" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3375,7 +3472,7 @@
           <t>PO14752942</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="B115" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3398,7 +3495,7 @@
           <t>PO16393493</t>
         </is>
       </c>
-      <c r="B116" s="4" t="inlineStr">
+      <c r="B116" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3421,7 +3518,7 @@
           <t>PO16450842</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B117" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3444,7 +3541,7 @@
           <t>PO16258342</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B118" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3467,7 +3564,7 @@
           <t>PO15682306</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B119" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3490,7 +3587,7 @@
           <t>PO16306253</t>
         </is>
       </c>
-      <c r="B120" s="4" t="inlineStr">
+      <c r="B120" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3513,7 +3610,7 @@
           <t>PO16339962</t>
         </is>
       </c>
-      <c r="B121" s="4" t="inlineStr">
+      <c r="B121" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3536,7 +3633,7 @@
           <t>PO16270912</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B122" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3559,7 +3656,7 @@
           <t>PO14769929</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr">
+      <c r="B123" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3582,7 +3679,7 @@
           <t>PO15785209</t>
         </is>
       </c>
-      <c r="B124" s="4" t="inlineStr">
+      <c r="B124" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3605,7 +3702,7 @@
           <t>PO16272511</t>
         </is>
       </c>
-      <c r="B125" s="4" t="inlineStr">
+      <c r="B125" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3628,7 +3725,7 @@
           <t>PO16301482</t>
         </is>
       </c>
-      <c r="B126" s="4" t="inlineStr">
+      <c r="B126" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3651,7 +3748,7 @@
           <t>PO15682293</t>
         </is>
       </c>
-      <c r="B127" s="4" t="inlineStr">
+      <c r="B127" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3674,7 +3771,7 @@
           <t>PO16413100</t>
         </is>
       </c>
-      <c r="B128" s="4" t="inlineStr">
+      <c r="B128" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3697,7 +3794,7 @@
           <t>PO16235990</t>
         </is>
       </c>
-      <c r="B129" s="4" t="inlineStr">
+      <c r="B129" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3720,7 +3817,7 @@
           <t>PO14769932</t>
         </is>
       </c>
-      <c r="B130" s="4" t="inlineStr">
+      <c r="B130" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3743,7 +3840,7 @@
           <t>PO16297395</t>
         </is>
       </c>
-      <c r="B131" s="4" t="inlineStr">
+      <c r="B131" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3766,7 +3863,7 @@
           <t>PO15014523</t>
         </is>
       </c>
-      <c r="B132" s="4" t="inlineStr">
+      <c r="B132" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3789,7 +3886,7 @@
           <t>PO16272686</t>
         </is>
       </c>
-      <c r="B133" s="4" t="inlineStr">
+      <c r="B133" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3812,7 +3909,7 @@
           <t>PO16333132</t>
         </is>
       </c>
-      <c r="B134" s="4" t="inlineStr">
+      <c r="B134" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3835,7 +3932,7 @@
           <t>PO16215842</t>
         </is>
       </c>
-      <c r="B135" s="4" t="inlineStr">
+      <c r="B135" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3858,7 +3955,7 @@
           <t>PO16498047</t>
         </is>
       </c>
-      <c r="B136" s="4" t="inlineStr">
+      <c r="B136" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3881,7 +3978,7 @@
           <t>PO16245570</t>
         </is>
       </c>
-      <c r="B137" s="4" t="inlineStr">
+      <c r="B137" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3904,7 +4001,7 @@
           <t>PO16402279</t>
         </is>
       </c>
-      <c r="B138" s="4" t="inlineStr">
+      <c r="B138" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3927,7 +4024,7 @@
           <t>PO16435058</t>
         </is>
       </c>
-      <c r="B139" s="4" t="inlineStr">
+      <c r="B139" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3950,7 +4047,7 @@
           <t>PO16413502</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B140" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3973,7 +4070,7 @@
           <t>PO16262207</t>
         </is>
       </c>
-      <c r="B141" s="4" t="inlineStr">
+      <c r="B141" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3996,7 +4093,7 @@
           <t>PO16206445</t>
         </is>
       </c>
-      <c r="B142" s="4" t="inlineStr">
+      <c r="B142" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4019,7 +4116,7 @@
           <t>PO16447332</t>
         </is>
       </c>
-      <c r="B143" s="4" t="inlineStr">
+      <c r="B143" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4042,7 +4139,7 @@
           <t>PO16253764</t>
         </is>
       </c>
-      <c r="B144" s="4" t="inlineStr">
+      <c r="B144" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4065,7 +4162,7 @@
           <t>PO16228701</t>
         </is>
       </c>
-      <c r="B145" s="4" t="inlineStr">
+      <c r="B145" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4088,7 +4185,7 @@
           <t>PO14752943</t>
         </is>
       </c>
-      <c r="B146" s="4" t="inlineStr">
+      <c r="B146" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4111,7 +4208,7 @@
           <t>PO16440218</t>
         </is>
       </c>
-      <c r="B147" s="4" t="inlineStr">
+      <c r="B147" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4134,7 +4231,7 @@
           <t>PO16004691</t>
         </is>
       </c>
-      <c r="B148" s="4" t="inlineStr">
+      <c r="B148" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4157,7 +4254,7 @@
           <t>PO16435620</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B149" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4180,7 +4277,7 @@
           <t>PO16366728</t>
         </is>
       </c>
-      <c r="B150" s="4" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4203,7 +4300,7 @@
           <t>PO14760860</t>
         </is>
       </c>
-      <c r="B151" s="4" t="inlineStr">
+      <c r="B151" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4226,7 +4323,7 @@
           <t>PO16428321</t>
         </is>
       </c>
-      <c r="B152" s="4" t="inlineStr">
+      <c r="B152" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4249,7 +4346,7 @@
           <t>PO16242875</t>
         </is>
       </c>
-      <c r="B153" s="4" t="inlineStr">
+      <c r="B153" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4272,7 +4369,7 @@
           <t>PO16555178</t>
         </is>
       </c>
-      <c r="B154" s="4" t="inlineStr">
+      <c r="B154" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4295,7 +4392,7 @@
           <t>PO16410925</t>
         </is>
       </c>
-      <c r="B155" s="4" t="inlineStr">
+      <c r="B155" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4318,7 +4415,7 @@
           <t>PO16230212</t>
         </is>
       </c>
-      <c r="B156" s="4" t="inlineStr">
+      <c r="B156" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4341,7 +4438,7 @@
           <t>PO16165759</t>
         </is>
       </c>
-      <c r="B157" s="4" t="inlineStr">
+      <c r="B157" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4364,7 +4461,7 @@
           <t>PO16575659</t>
         </is>
       </c>
-      <c r="B158" s="4" t="inlineStr">
+      <c r="B158" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4387,7 +4484,7 @@
           <t>PO14034238</t>
         </is>
       </c>
-      <c r="B159" s="4" t="inlineStr">
+      <c r="B159" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4410,7 +4507,7 @@
           <t>PO16388003</t>
         </is>
       </c>
-      <c r="B160" s="4" t="inlineStr">
+      <c r="B160" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4433,7 +4530,7 @@
           <t>PO16569182</t>
         </is>
       </c>
-      <c r="B161" s="4" t="inlineStr">
+      <c r="B161" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4456,7 +4553,7 @@
           <t>PO16501867</t>
         </is>
       </c>
-      <c r="B162" s="4" t="inlineStr">
+      <c r="B162" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4479,7 +4576,7 @@
           <t>PO16390572</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
+      <c r="B163" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4502,7 +4599,7 @@
           <t>PO16541834</t>
         </is>
       </c>
-      <c r="B164" s="4" t="inlineStr">
+      <c r="B164" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4525,7 +4622,7 @@
           <t>PO14752925</t>
         </is>
       </c>
-      <c r="B165" s="4" t="inlineStr">
+      <c r="B165" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4548,7 +4645,7 @@
           <t>PO16435057</t>
         </is>
       </c>
-      <c r="B166" s="4" t="inlineStr">
+      <c r="B166" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4571,7 +4668,7 @@
           <t>PO16512210</t>
         </is>
       </c>
-      <c r="B167" s="4" t="inlineStr">
+      <c r="B167" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4594,7 +4691,7 @@
           <t>PO16386814</t>
         </is>
       </c>
-      <c r="B168" s="4" t="inlineStr">
+      <c r="B168" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4617,7 +4714,7 @@
           <t>PO16321781</t>
         </is>
       </c>
-      <c r="B169" s="4" t="inlineStr">
+      <c r="B169" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4640,7 +4737,7 @@
           <t>PO16255601</t>
         </is>
       </c>
-      <c r="B170" s="4" t="inlineStr">
+      <c r="B170" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4663,7 +4760,7 @@
           <t>PO16355659</t>
         </is>
       </c>
-      <c r="B171" s="4" t="inlineStr">
+      <c r="B171" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4686,7 +4783,7 @@
           <t>PO16489207</t>
         </is>
       </c>
-      <c r="B172" s="4" t="inlineStr">
+      <c r="B172" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4709,7 +4806,7 @@
           <t>PO15699499</t>
         </is>
       </c>
-      <c r="B173" s="4" t="inlineStr">
+      <c r="B173" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4732,7 +4829,7 @@
           <t>PO13622314</t>
         </is>
       </c>
-      <c r="B174" s="4" t="inlineStr">
+      <c r="B174" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4755,7 +4852,7 @@
           <t>PO15429046</t>
         </is>
       </c>
-      <c r="B175" s="4" t="inlineStr">
+      <c r="B175" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4778,7 +4875,7 @@
           <t>PO16394533</t>
         </is>
       </c>
-      <c r="B176" s="4" t="inlineStr">
+      <c r="B176" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4801,7 +4898,7 @@
           <t>PO16455498</t>
         </is>
       </c>
-      <c r="B177" s="4" t="inlineStr">
+      <c r="B177" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4824,7 +4921,7 @@
           <t>PO16326521</t>
         </is>
       </c>
-      <c r="B178" s="4" t="inlineStr">
+      <c r="B178" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4847,7 +4944,7 @@
           <t>PO15630092</t>
         </is>
       </c>
-      <c r="B179" s="4" t="inlineStr">
+      <c r="B179" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4870,7 +4967,7 @@
           <t>PO16433571</t>
         </is>
       </c>
-      <c r="B180" s="4" t="inlineStr">
+      <c r="B180" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4893,7 +4990,7 @@
           <t>PO16341901</t>
         </is>
       </c>
-      <c r="B181" s="4" t="inlineStr">
+      <c r="B181" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4916,7 +5013,7 @@
           <t>PO16064431</t>
         </is>
       </c>
-      <c r="B182" s="4" t="inlineStr">
+      <c r="B182" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4939,7 +5036,7 @@
           <t>PO14219870</t>
         </is>
       </c>
-      <c r="B183" s="4" t="inlineStr">
+      <c r="B183" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4962,7 +5059,7 @@
           <t>PO15630214</t>
         </is>
       </c>
-      <c r="B184" s="4" t="inlineStr">
+      <c r="B184" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4985,7 +5082,7 @@
           <t>PO15644153</t>
         </is>
       </c>
-      <c r="B185" s="4" t="inlineStr">
+      <c r="B185" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5008,7 +5105,7 @@
           <t>PO16256064</t>
         </is>
       </c>
-      <c r="B186" s="4" t="inlineStr">
+      <c r="B186" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5031,7 +5128,7 @@
           <t>PO15647942</t>
         </is>
       </c>
-      <c r="B187" s="4" t="inlineStr">
+      <c r="B187" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5054,7 +5151,7 @@
           <t>PO16322639</t>
         </is>
       </c>
-      <c r="B188" s="4" t="inlineStr">
+      <c r="B188" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5077,7 +5174,7 @@
           <t>PO16329589</t>
         </is>
       </c>
-      <c r="B189" s="4" t="inlineStr">
+      <c r="B189" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5100,7 +5197,7 @@
           <t>PO16184045</t>
         </is>
       </c>
-      <c r="B190" s="4" t="inlineStr">
+      <c r="B190" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5123,7 +5220,7 @@
           <t>PO16495607</t>
         </is>
       </c>
-      <c r="B191" s="4" t="inlineStr">
+      <c r="B191" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5146,7 +5243,7 @@
           <t>PO16438043</t>
         </is>
       </c>
-      <c r="B192" s="4" t="inlineStr">
+      <c r="B192" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5169,7 +5266,7 @@
           <t>PO15014528</t>
         </is>
       </c>
-      <c r="B193" s="4" t="inlineStr">
+      <c r="B193" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5192,7 +5289,7 @@
           <t>PO16299456</t>
         </is>
       </c>
-      <c r="B194" s="4" t="inlineStr">
+      <c r="B194" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5215,7 +5312,7 @@
           <t>PO16433499</t>
         </is>
       </c>
-      <c r="B195" s="4" t="inlineStr">
+      <c r="B195" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5238,7 +5335,7 @@
           <t>PO16441737</t>
         </is>
       </c>
-      <c r="B196" s="4" t="inlineStr">
+      <c r="B196" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5261,7 +5358,7 @@
           <t>PO15694769</t>
         </is>
       </c>
-      <c r="B197" s="4" t="inlineStr">
+      <c r="B197" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5284,7 +5381,7 @@
           <t>PO15694772</t>
         </is>
       </c>
-      <c r="B198" s="4" t="inlineStr">
+      <c r="B198" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5307,7 +5404,7 @@
           <t>PO16496851</t>
         </is>
       </c>
-      <c r="B199" s="4" t="inlineStr">
+      <c r="B199" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5330,7 +5427,7 @@
           <t>PO13653137</t>
         </is>
       </c>
-      <c r="B200" s="4" t="inlineStr">
+      <c r="B200" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5353,7 +5450,7 @@
           <t>PO16389062</t>
         </is>
       </c>
-      <c r="B201" s="4" t="inlineStr">
+      <c r="B201" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5376,7 +5473,7 @@
           <t>PO15695018</t>
         </is>
       </c>
-      <c r="B202" s="4" t="inlineStr">
+      <c r="B202" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5399,7 +5496,7 @@
           <t>PO16152224</t>
         </is>
       </c>
-      <c r="B203" s="4" t="inlineStr">
+      <c r="B203" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5422,7 +5519,7 @@
           <t>PO16511466</t>
         </is>
       </c>
-      <c r="B204" s="4" t="inlineStr">
+      <c r="B204" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5445,7 +5542,7 @@
           <t>PO16191221</t>
         </is>
       </c>
-      <c r="B205" s="4" t="inlineStr">
+      <c r="B205" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5468,7 +5565,7 @@
           <t>PO14752926</t>
         </is>
       </c>
-      <c r="B206" s="4" t="inlineStr">
+      <c r="B206" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5491,7 +5588,7 @@
           <t>PO15628885</t>
         </is>
       </c>
-      <c r="B207" s="4" t="inlineStr">
+      <c r="B207" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5514,7 +5611,7 @@
           <t>PO16314188</t>
         </is>
       </c>
-      <c r="B208" s="4" t="inlineStr">
+      <c r="B208" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5537,7 +5634,7 @@
           <t>PO14607065</t>
         </is>
       </c>
-      <c r="B209" s="4" t="inlineStr">
+      <c r="B209" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5560,7 +5657,7 @@
           <t>PO16064432</t>
         </is>
       </c>
-      <c r="B210" s="4" t="inlineStr">
+      <c r="B210" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5583,7 +5680,7 @@
           <t>PO16340514</t>
         </is>
       </c>
-      <c r="B211" s="4" t="inlineStr">
+      <c r="B211" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5606,7 +5703,7 @@
           <t>PO16006846</t>
         </is>
       </c>
-      <c r="B212" s="4" t="inlineStr">
+      <c r="B212" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5629,7 +5726,7 @@
           <t>PO15630301</t>
         </is>
       </c>
-      <c r="B213" s="4" t="inlineStr">
+      <c r="B213" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5652,7 +5749,7 @@
           <t>PO16243291</t>
         </is>
       </c>
-      <c r="B214" s="4" t="inlineStr">
+      <c r="B214" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5675,7 +5772,7 @@
           <t>PO16450524</t>
         </is>
       </c>
-      <c r="B215" s="4" t="inlineStr">
+      <c r="B215" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5698,7 +5795,7 @@
           <t>PO16518287</t>
         </is>
       </c>
-      <c r="B216" s="4" t="inlineStr">
+      <c r="B216" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5721,7 +5818,7 @@
           <t>PO16501626</t>
         </is>
       </c>
-      <c r="B217" s="4" t="inlineStr">
+      <c r="B217" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5744,7 +5841,7 @@
           <t>PO14065853</t>
         </is>
       </c>
-      <c r="B218" s="4" t="inlineStr">
+      <c r="B218" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5767,7 +5864,7 @@
           <t>PO15694770</t>
         </is>
       </c>
-      <c r="B219" s="4" t="inlineStr">
+      <c r="B219" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5790,7 +5887,7 @@
           <t>PO16501625</t>
         </is>
       </c>
-      <c r="B220" s="4" t="inlineStr">
+      <c r="B220" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5813,7 +5910,7 @@
           <t>PO16396709</t>
         </is>
       </c>
-      <c r="B221" s="4" t="inlineStr">
+      <c r="B221" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5836,7 +5933,7 @@
           <t>PO16404433</t>
         </is>
       </c>
-      <c r="B222" s="4" t="inlineStr">
+      <c r="B222" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5859,7 +5956,7 @@
           <t>PO16356881</t>
         </is>
       </c>
-      <c r="B223" s="4" t="inlineStr">
+      <c r="B223" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5882,7 +5979,7 @@
           <t>PO15694761</t>
         </is>
       </c>
-      <c r="B224" s="4" t="inlineStr">
+      <c r="B224" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5905,7 +6002,7 @@
           <t>PO15613054</t>
         </is>
       </c>
-      <c r="B225" s="4" t="inlineStr">
+      <c r="B225" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5928,7 +6025,7 @@
           <t>PO15630315</t>
         </is>
       </c>
-      <c r="B226" s="4" t="inlineStr">
+      <c r="B226" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5951,7 +6048,7 @@
           <t>PO15694762</t>
         </is>
       </c>
-      <c r="B227" s="4" t="inlineStr">
+      <c r="B227" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5974,7 +6071,7 @@
           <t>PO16370804</t>
         </is>
       </c>
-      <c r="B228" s="4" t="inlineStr">
+      <c r="B228" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5997,7 +6094,7 @@
           <t>PO16145734</t>
         </is>
       </c>
-      <c r="B229" s="4" t="inlineStr">
+      <c r="B229" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6020,7 +6117,7 @@
           <t>PO16361280</t>
         </is>
       </c>
-      <c r="B230" s="4" t="inlineStr">
+      <c r="B230" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6043,7 +6140,7 @@
           <t>PO15699771</t>
         </is>
       </c>
-      <c r="B231" s="4" t="inlineStr">
+      <c r="B231" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6066,7 +6163,7 @@
           <t>PO16362352</t>
         </is>
       </c>
-      <c r="B232" s="4" t="inlineStr">
+      <c r="B232" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6089,7 +6186,7 @@
           <t>PO16530239</t>
         </is>
       </c>
-      <c r="B233" s="4" t="inlineStr">
+      <c r="B233" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6112,7 +6209,7 @@
           <t>PO16051893</t>
         </is>
       </c>
-      <c r="B234" s="4" t="inlineStr">
+      <c r="B234" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6135,7 +6232,7 @@
           <t>PO16330375</t>
         </is>
       </c>
-      <c r="B235" s="4" t="inlineStr">
+      <c r="B235" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6158,7 +6255,7 @@
           <t>PO15241466</t>
         </is>
       </c>
-      <c r="B236" s="4" t="inlineStr">
+      <c r="B236" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6181,7 +6278,7 @@
           <t>PO16442571</t>
         </is>
       </c>
-      <c r="B237" s="4" t="inlineStr">
+      <c r="B237" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6204,7 +6301,7 @@
           <t>PO16157599</t>
         </is>
       </c>
-      <c r="B238" s="4" t="inlineStr">
+      <c r="B238" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6227,7 +6324,7 @@
           <t>PO14738382</t>
         </is>
       </c>
-      <c r="B239" s="4" t="inlineStr">
+      <c r="B239" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6250,7 +6347,7 @@
           <t>PO14760883</t>
         </is>
       </c>
-      <c r="B240" s="4" t="inlineStr">
+      <c r="B240" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6273,7 +6370,7 @@
           <t>PO14719278</t>
         </is>
       </c>
-      <c r="B241" s="4" t="inlineStr">
+      <c r="B241" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6296,7 +6393,7 @@
           <t>PO14760850</t>
         </is>
       </c>
-      <c r="B242" s="4" t="inlineStr">
+      <c r="B242" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6319,7 +6416,7 @@
           <t>PO14719338</t>
         </is>
       </c>
-      <c r="B243" s="4" t="inlineStr">
+      <c r="B243" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6342,7 +6439,7 @@
           <t>PO16359448</t>
         </is>
       </c>
-      <c r="B244" s="4" t="inlineStr">
+      <c r="B244" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6365,7 +6462,7 @@
           <t>PO16547176</t>
         </is>
       </c>
-      <c r="B245" s="4" t="inlineStr">
+      <c r="B245" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6388,7 +6485,7 @@
           <t>PO14010216</t>
         </is>
       </c>
-      <c r="B246" s="4" t="inlineStr">
+      <c r="B246" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6411,7 +6508,7 @@
           <t>PO14010221</t>
         </is>
       </c>
-      <c r="B247" s="4" t="inlineStr">
+      <c r="B247" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6434,7 +6531,7 @@
           <t>PO16323002</t>
         </is>
       </c>
-      <c r="B248" s="4" t="inlineStr">
+      <c r="B248" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6457,7 +6554,7 @@
           <t>PO16315115</t>
         </is>
       </c>
-      <c r="B249" s="4" t="inlineStr">
+      <c r="B249" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6480,7 +6577,7 @@
           <t>PO16488717</t>
         </is>
       </c>
-      <c r="B250" s="4" t="inlineStr">
+      <c r="B250" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6503,7 +6600,7 @@
           <t>PO16522171</t>
         </is>
       </c>
-      <c r="B251" s="4" t="inlineStr">
+      <c r="B251" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6526,7 +6623,7 @@
           <t>PO16485947</t>
         </is>
       </c>
-      <c r="B252" s="4" t="inlineStr">
+      <c r="B252" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6549,7 +6646,7 @@
           <t>PO15874912</t>
         </is>
       </c>
-      <c r="B253" s="4" t="inlineStr">
+      <c r="B253" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6572,7 +6669,7 @@
           <t>PO13064901</t>
         </is>
       </c>
-      <c r="B254" s="4" t="inlineStr">
+      <c r="B254" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6595,7 +6692,7 @@
           <t>PO15614578</t>
         </is>
       </c>
-      <c r="B255" s="4" t="inlineStr">
+      <c r="B255" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6618,7 +6715,7 @@
           <t>PO16224336</t>
         </is>
       </c>
-      <c r="B256" s="4" t="inlineStr">
+      <c r="B256" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6641,7 +6738,7 @@
           <t>PO16207339</t>
         </is>
       </c>
-      <c r="B257" s="4" t="inlineStr">
+      <c r="B257" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6664,7 +6761,7 @@
           <t>PO14010218</t>
         </is>
       </c>
-      <c r="B258" s="4" t="inlineStr">
+      <c r="B258" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6687,7 +6784,7 @@
           <t>PO16202587</t>
         </is>
       </c>
-      <c r="B259" s="4" t="inlineStr">
+      <c r="B259" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6710,7 +6807,7 @@
           <t>PO16211797</t>
         </is>
       </c>
-      <c r="B260" s="4" t="inlineStr">
+      <c r="B260" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6733,7 +6830,7 @@
           <t>PO15220371</t>
         </is>
       </c>
-      <c r="B261" s="4" t="inlineStr">
+      <c r="B261" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6756,7 +6853,7 @@
           <t>PO16271627</t>
         </is>
       </c>
-      <c r="B262" s="4" t="inlineStr">
+      <c r="B262" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6779,7 +6876,7 @@
           <t>PO16264130</t>
         </is>
       </c>
-      <c r="B263" s="4" t="inlineStr">
+      <c r="B263" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6802,7 +6899,7 @@
           <t>PO14008887</t>
         </is>
       </c>
-      <c r="B264" s="4" t="inlineStr">
+      <c r="B264" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6825,7 +6922,7 @@
           <t>PO14958078</t>
         </is>
       </c>
-      <c r="B265" s="4" t="inlineStr">
+      <c r="B265" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6848,7 +6945,7 @@
           <t>PO13406596</t>
         </is>
       </c>
-      <c r="B266" s="4" t="inlineStr">
+      <c r="B266" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6871,7 +6968,7 @@
           <t>PO15220377</t>
         </is>
       </c>
-      <c r="B267" s="4" t="inlineStr">
+      <c r="B267" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6894,7 +6991,7 @@
           <t>PO13247181</t>
         </is>
       </c>
-      <c r="B268" s="4" t="inlineStr">
+      <c r="B268" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>

</xml_diff>

<commit_message>
feat(security): add comprehensive security features and digital signatures
- Add security_setup.py for digital signature and security features
- Implement self-signed certificate creation for code signing
- Add security checksums (MD5/SHA256) for file integrity verification
- Create security manifest for Windows compatibility
- Add version information and professional metadata
- Implement PyInstaller security optimizations (strip, UPX, excludes)
- Add comprehensive security documentation (SECURITY.md)
- Update build_single_exe.py with security enhancements
- Add security section to README with troubleshooting guide
- Include Windows Defender and SmartScreen compatibility measures

Security features:
- Digital signature with timestamp server
- File integrity checksums
- Professional metadata and version info
- Security manifest for Windows
- Optimized build to avoid false positives
- Comprehensive security documentation
- Verification instructions for users
</commit_message>
<xml_diff>
--- a/data/input/input.xlsx
+++ b/data/input/input.xlsx
@@ -544,9 +544,9 @@
           <t>PO16400507</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -558,11 +558,11 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025-08-04 23:38:49</t>
+          <t>2025-08-04 23:55:27</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -597,7 +597,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-08-04 23:38:50</t>
+          <t>2025-08-05 00:12:30</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -614,9 +614,9 @@
           <t>PO15377448</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -628,11 +628,11 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2025-08-04 23:39:01</t>
+          <t>2025-08-05 00:12:48</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -887,9 +887,9 @@
           <t>PO15682304</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -901,11 +901,11 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-08-04 23:39:12</t>
+          <t>2025-08-05 00:13:06</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-08-04 23:39:23</t>
+          <t>2025-08-05 00:13:19</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025-08-04 23:39:49</t>
+          <t>2025-08-05 00:13:20</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1308,9 +1308,9 @@
           <t>PO15345517</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1322,11 +1322,11 @@
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2025-08-04 23:40:03</t>
+          <t>2025-08-05 00:13:35</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1425,22 +1425,38 @@
           <t>PO16370617</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cornerstone_OnDemand_Limited-0050436383</t>
+        </is>
+      </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:13:59</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Cornerstone_OnDemand_Limited-0050436383/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16370617</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1448,22 +1464,38 @@
           <t>PO15776178</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PROJECT_ONE_CONSULTING_LIMITED-0051463283</t>
+        </is>
+      </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:14:16</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>PROJECT_ONE_CONSULTING_LIMITED-0051463283/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15776178</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1471,22 +1503,38 @@
           <t>PO16110682</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>NIIT_LIMITED_UK-0001095749</t>
+        </is>
+      </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:49:56</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NIIT_LIMITED_UK-0001095749/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16110682</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1494,22 +1542,38 @@
           <t>PO16295766</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>THOUCENTRIC_LIMITED-0050540063</t>
+        </is>
+      </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:04</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>THOUCENTRIC_LIMITED-0050540063/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16295766</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1517,22 +1581,38 @@
           <t>PO16263753</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LTIMINDTREE_LIMITED-0051615301</t>
+        </is>
+      </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:12</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>LTIMINDTREE_LIMITED-0051615301/</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16263753</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1540,22 +1620,38 @@
           <t>PO16243786</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>HCL_TECHNOLOGIES_UK_LTD-0050483341</t>
+        </is>
+      </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:21</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>HCL_TECHNOLOGIES_UK_LTD-0050483341/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16243786</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1563,22 +1659,38 @@
           <t>PO15190568</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ROGERS-0050276068</t>
+        </is>
+      </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:33</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ROGERS-0050276068/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15190568</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1586,9 +1698,9 @@
           <t>PO15279299</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NO_ATTACHMENTS</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1598,10 +1710,18 @@
       <c r="E33" t="n">
         <v>0</v>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:14:18</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15279299</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1609,22 +1729,38 @@
           <t>PO16311692</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312</t>
+        </is>
+      </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:43</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16311692</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1632,22 +1768,38 @@
           <t>PO16508611</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PRICEWATERHOUSECOOPERS_PRIVATE_LIMITED-0050437782</t>
+        </is>
+      </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:50:55</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>PRICEWATERHOUSECOOPERS_PRIVATE_LIMITED-0050437782/</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16508611</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1655,22 +1807,38 @@
           <t>PO16291902</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001016941</t>
+        </is>
+      </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:51:06</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001016941/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16291902</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1678,22 +1846,38 @@
           <t>PO16291905</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001016941</t>
+        </is>
+      </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:51:17</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001016941/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16291905</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1701,22 +1885,38 @@
           <t>PO16362026</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ernst_and_Young_LLP-0051619549</t>
+        </is>
+      </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:14:36</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Ernst_and_Young_LLP-0051619549/</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16362026</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1724,22 +1924,38 @@
           <t>PO16401398</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BIRLASOFT_SOLUTIONS_LIMITED-0000230143</t>
+        </is>
+      </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:51:51</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>BIRLASOFT_SOLUTIONS_LIMITED-0000230143/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16401398</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1747,22 +1963,38 @@
           <t>PO16258825</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>COGNIZANT_WORLDWIDE_LTD_UK_LTD-0001100952</t>
+        </is>
+      </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2025-08-04 23:52:03</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>COGNIZANT_WORLDWIDE_LTD_UK_LTD-0001100952/</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16258825</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1770,22 +2002,38 @@
           <t>PO16329900</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>RESOURCES_CONNECTION_UK_LTD_RESOURCES_GLOBAL_PROFESSIONALS-0001039917</t>
+        </is>
+      </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:14:48</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>RESOURCES_CONNECTION_UK_LTD_RESOURCES_GLOBAL_PROFESSIONALS-0001039917/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16329900</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1793,22 +2041,38 @@
           <t>PO16307414</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>JK_TECHNOSOFT_LTD-0050231277</t>
+        </is>
+      </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:14:59</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>JK_TECHNOSOFT_LTD-0050231277/</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16307414</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1816,9 +2080,9 @@
           <t>PO15910712</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NO_ATTACHMENTS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1828,10 +2092,18 @@
       <c r="E43" t="n">
         <v>0</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:15:02</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15910712</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1839,22 +2111,38 @@
           <t>PO16323977</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312</t>
+        </is>
+      </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:15:16</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312/</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16323977</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">

</xml_diff>

<commit_message>
feat(excel-workflow): add Excel-based input workflow with template
- Add build_single_exe_excel_workflow.py for Excel-based EXE
- Create Excel template with headers and sample data
- Implement workflow: open template → user edits → save → process
- Add temporary workspace management
- Integrate with original download system
- Move processed files to Downloads/CoupaDownloads/
- Add comprehensive instructions and validation
- Support both Excel (.xlsx) and CSV formats
- Include professional template styling and instructions sheet

Excel workflow features:
- Professional Excel template with headers
- Sample data and instructions sheet
- Temporary workspace creation
- Automatic file opening and processing
- Integration with original system
- Move to downloads folder after completion
- Progress tracking and validation
</commit_message>
<xml_diff>
--- a/data/input/input.xlsx
+++ b/data/input/input.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-08-05 00:12:30</t>
+          <t>2025-08-05 00:26:55</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-08-05 00:13:19</t>
+          <t>2025-08-05 00:27:06</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025-08-05 00:13:20</t>
+          <t>2025-08-05 00:27:06</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2025-08-05 00:13:59</t>
+          <t>2025-08-05 00:27:30</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2025-08-05 00:14:16</t>
+          <t>2025-08-05 00:27:48</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2025-08-05 00:14:18</t>
+          <t>2025-08-05 00:27:50</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2025-08-05 00:14:36</t>
+          <t>2025-08-05 00:28:08</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2025-08-05 00:14:48</t>
+          <t>2025-08-05 00:28:19</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2025-08-05 00:15:02</t>
+          <t>2025-08-05 00:28:21</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2150,22 +2150,38 @@
           <t>PO16400408</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CONNECTED_IT_CONTRACT_LIMITED-0050547915</t>
+        </is>
+      </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:28:29</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>CONNECTED_IT_CONTRACT_LIMITED-0050547915/</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16400408</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2173,22 +2189,38 @@
           <t>PO16359621</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>DELOITTE_TOUCHE_TOHMATSU_INDIA_LLP-0050532353</t>
+        </is>
+      </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:28:36</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>DELOITTE_TOUCHE_TOHMATSU_INDIA_LLP-0050532353/</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16359621</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2196,22 +2228,38 @@
           <t>PO16242475</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312</t>
+        </is>
+      </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:28:51</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>ERNST_AND_YOUNG_LLP-0001118312/</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/16242475</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2219,9 +2267,9 @@
           <t>PO15436910</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>NO_ATTACHMENTS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2231,10 +2279,18 @@
       <c r="E48" t="n">
         <v>0</v>
       </c>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:28:51</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15436910</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2242,9 +2298,9 @@
           <t>PO15179449</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>NO_ATTACHMENTS</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2254,10 +2310,18 @@
       <c r="E49" t="n">
         <v>0</v>
       </c>
-      <c r="F49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2025-08-05 00:28:52</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://unilever.coupahost.com/order_headers/15179449</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">

</xml_diff>

<commit_message>
refactor: remove outdated build scripts and add new GitHub release preparation script
- Deleted legacy build scripts for EXE and portable package creation.
- Introduced create_github_release.py for streamlined release preparation.
- Added comprehensive documentation for EdgeDriver 138 bundle and troubleshooting.
- Updated project structure to enhance maintainability and user experience.
</commit_message>
<xml_diff>
--- a/data/input/input.xlsx
+++ b/data/input/input.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0090EE90"/>
         <bgColor rgb="0090EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB6C1"/>
+        <bgColor rgb="00FFB6C1"/>
       </patternFill>
     </fill>
     <fill>
@@ -77,13 +83,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -597,7 +604,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-08-05 00:53:28</t>
+          <t>2025-08-05 08:55:57</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -965,9 +972,9 @@
           <t>PO14174358</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -979,11 +986,11 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-08-05 00:53:40</t>
+          <t>2025-08-05 05:01:30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1291,7 +1298,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025-08-05 00:53:41</t>
+          <t>2025-08-05 05:01:31</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1443,7 +1450,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2025-08-05 00:54:04</t>
+          <t>2025-08-05 05:01:54</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1482,7 +1489,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2025-08-05 00:54:22</t>
+          <t>2025-08-05 05:02:33</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1712,7 +1719,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2025-08-05 00:54:24</t>
+          <t>2025-08-05 05:02:35</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -1903,7 +1910,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2025-08-05 00:54:41</t>
+          <t>2025-08-05 05:02:52</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2586,7 +2593,7 @@
           <t>PO16407260</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2609,7 +2616,7 @@
           <t>PO16353483</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2632,7 +2639,7 @@
           <t>PO15287725</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2655,7 +2662,7 @@
           <t>PO16413103</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2678,7 +2685,7 @@
           <t>PO16465704</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2701,7 +2708,7 @@
           <t>PO16510823</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2724,7 +2731,7 @@
           <t>PO16224968</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2747,7 +2754,7 @@
           <t>PO16556376</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2770,7 +2777,7 @@
           <t>PO16488279</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2793,7 +2800,7 @@
           <t>PO15630093</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2816,7 +2823,7 @@
           <t>PO16262209</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2839,7 +2846,7 @@
           <t>PO16477243</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2862,7 +2869,7 @@
           <t>PO15617175</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2885,7 +2892,7 @@
           <t>PO16384342</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2908,7 +2915,7 @@
           <t>PO15285778</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2931,7 +2938,7 @@
           <t>PO16398622</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2954,7 +2961,7 @@
           <t>PO15154338</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -2977,7 +2984,7 @@
           <t>PO16207336</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3000,7 +3007,7 @@
           <t>PO16269922</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3023,7 +3030,7 @@
           <t>PO16400435</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3046,7 +3053,7 @@
           <t>PO16264501</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3069,7 +3076,7 @@
           <t>PO14729307</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3092,7 +3099,7 @@
           <t>PO16105473</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3115,7 +3122,7 @@
           <t>PO15437050</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3138,7 +3145,7 @@
           <t>PO15617177</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3161,7 +3168,7 @@
           <t>PO16497039</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3184,7 +3191,7 @@
           <t>PO16400407</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3207,7 +3214,7 @@
           <t>PO16219761</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3230,7 +3237,7 @@
           <t>PO15694773</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3253,7 +3260,7 @@
           <t>PO16539229</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3276,7 +3283,7 @@
           <t>PO16233980</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3299,7 +3306,7 @@
           <t>PO13068435</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3322,7 +3329,7 @@
           <t>PO16366575</t>
         </is>
       </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3345,7 +3352,7 @@
           <t>PO16343173</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3368,7 +3375,7 @@
           <t>PO16253759</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3391,7 +3398,7 @@
           <t>PO15285775</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3414,7 +3421,7 @@
           <t>PO16240302</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3437,7 +3444,7 @@
           <t>PO14752945</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3460,7 +3467,7 @@
           <t>PO16393498</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3483,7 +3490,7 @@
           <t>PO13081743</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3506,7 +3513,7 @@
           <t>PO15617218</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3529,7 +3536,7 @@
           <t>PO15285806</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3552,7 +3559,7 @@
           <t>PO16253702</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3575,7 +3582,7 @@
           <t>PO16330407</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3598,7 +3605,7 @@
           <t>PO16322561</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3621,7 +3628,7 @@
           <t>PO13019654</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3644,7 +3651,7 @@
           <t>PO16188865</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B103" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3667,7 +3674,7 @@
           <t>PO15715793</t>
         </is>
       </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3690,7 +3697,7 @@
           <t>PO16380788</t>
         </is>
       </c>
-      <c r="B105" s="3" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3713,7 +3720,7 @@
           <t>PO16258716</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3736,7 +3743,7 @@
           <t>PO16191725</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3759,7 +3766,7 @@
           <t>PO15718023</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B108" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3782,7 +3789,7 @@
           <t>PO16258379</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B109" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3805,7 +3812,7 @@
           <t>PO14769933</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3828,7 +3835,7 @@
           <t>PO15980633</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3851,7 +3858,7 @@
           <t>PO16383021</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3874,7 +3881,7 @@
           <t>PO14769930</t>
         </is>
       </c>
-      <c r="B113" s="3" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3897,7 +3904,7 @@
           <t>PO16042562</t>
         </is>
       </c>
-      <c r="B114" s="3" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3920,7 +3927,7 @@
           <t>PO14752942</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3943,7 +3950,7 @@
           <t>PO16393493</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3966,7 +3973,7 @@
           <t>PO16450842</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -3989,7 +3996,7 @@
           <t>PO16258342</t>
         </is>
       </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4012,7 +4019,7 @@
           <t>PO15682306</t>
         </is>
       </c>
-      <c r="B119" s="3" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4035,7 +4042,7 @@
           <t>PO16306253</t>
         </is>
       </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4058,7 +4065,7 @@
           <t>PO16339962</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4081,7 +4088,7 @@
           <t>PO16270912</t>
         </is>
       </c>
-      <c r="B122" s="3" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4104,7 +4111,7 @@
           <t>PO14769929</t>
         </is>
       </c>
-      <c r="B123" s="3" t="inlineStr">
+      <c r="B123" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4127,7 +4134,7 @@
           <t>PO15785209</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4150,7 +4157,7 @@
           <t>PO16272511</t>
         </is>
       </c>
-      <c r="B125" s="3" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4173,7 +4180,7 @@
           <t>PO16301482</t>
         </is>
       </c>
-      <c r="B126" s="3" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4196,7 +4203,7 @@
           <t>PO15682293</t>
         </is>
       </c>
-      <c r="B127" s="3" t="inlineStr">
+      <c r="B127" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4219,7 +4226,7 @@
           <t>PO16413100</t>
         </is>
       </c>
-      <c r="B128" s="3" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4242,7 +4249,7 @@
           <t>PO16235990</t>
         </is>
       </c>
-      <c r="B129" s="3" t="inlineStr">
+      <c r="B129" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4265,7 +4272,7 @@
           <t>PO14769932</t>
         </is>
       </c>
-      <c r="B130" s="3" t="inlineStr">
+      <c r="B130" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4288,7 +4295,7 @@
           <t>PO16297395</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
+      <c r="B131" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4311,7 +4318,7 @@
           <t>PO15014523</t>
         </is>
       </c>
-      <c r="B132" s="3" t="inlineStr">
+      <c r="B132" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4334,7 +4341,7 @@
           <t>PO16272686</t>
         </is>
       </c>
-      <c r="B133" s="3" t="inlineStr">
+      <c r="B133" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4357,7 +4364,7 @@
           <t>PO16333132</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4380,7 +4387,7 @@
           <t>PO16215842</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr">
+      <c r="B135" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4403,7 +4410,7 @@
           <t>PO16498047</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr">
+      <c r="B136" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4426,7 +4433,7 @@
           <t>PO16245570</t>
         </is>
       </c>
-      <c r="B137" s="3" t="inlineStr">
+      <c r="B137" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4449,7 +4456,7 @@
           <t>PO16402279</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr">
+      <c r="B138" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4472,7 +4479,7 @@
           <t>PO16435058</t>
         </is>
       </c>
-      <c r="B139" s="3" t="inlineStr">
+      <c r="B139" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4495,7 +4502,7 @@
           <t>PO16413502</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="B140" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4518,7 +4525,7 @@
           <t>PO16262207</t>
         </is>
       </c>
-      <c r="B141" s="3" t="inlineStr">
+      <c r="B141" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4541,7 +4548,7 @@
           <t>PO16206445</t>
         </is>
       </c>
-      <c r="B142" s="3" t="inlineStr">
+      <c r="B142" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4564,7 +4571,7 @@
           <t>PO16447332</t>
         </is>
       </c>
-      <c r="B143" s="3" t="inlineStr">
+      <c r="B143" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4587,7 +4594,7 @@
           <t>PO16253764</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr">
+      <c r="B144" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4610,7 +4617,7 @@
           <t>PO16228701</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4633,7 +4640,7 @@
           <t>PO14752943</t>
         </is>
       </c>
-      <c r="B146" s="3" t="inlineStr">
+      <c r="B146" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4656,7 +4663,7 @@
           <t>PO16440218</t>
         </is>
       </c>
-      <c r="B147" s="3" t="inlineStr">
+      <c r="B147" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4679,7 +4686,7 @@
           <t>PO16004691</t>
         </is>
       </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="B148" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4702,7 +4709,7 @@
           <t>PO16435620</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B149" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4725,7 +4732,7 @@
           <t>PO16366728</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B150" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4748,7 +4755,7 @@
           <t>PO14760860</t>
         </is>
       </c>
-      <c r="B151" s="3" t="inlineStr">
+      <c r="B151" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4771,7 +4778,7 @@
           <t>PO16428321</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr">
+      <c r="B152" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4794,7 +4801,7 @@
           <t>PO16242875</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr">
+      <c r="B153" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4817,7 +4824,7 @@
           <t>PO16555178</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr">
+      <c r="B154" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4840,7 +4847,7 @@
           <t>PO16410925</t>
         </is>
       </c>
-      <c r="B155" s="3" t="inlineStr">
+      <c r="B155" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4863,7 +4870,7 @@
           <t>PO16230212</t>
         </is>
       </c>
-      <c r="B156" s="3" t="inlineStr">
+      <c r="B156" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4886,7 +4893,7 @@
           <t>PO16165759</t>
         </is>
       </c>
-      <c r="B157" s="3" t="inlineStr">
+      <c r="B157" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4909,7 +4916,7 @@
           <t>PO16575659</t>
         </is>
       </c>
-      <c r="B158" s="3" t="inlineStr">
+      <c r="B158" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4932,7 +4939,7 @@
           <t>PO14034238</t>
         </is>
       </c>
-      <c r="B159" s="3" t="inlineStr">
+      <c r="B159" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4955,7 +4962,7 @@
           <t>PO16388003</t>
         </is>
       </c>
-      <c r="B160" s="3" t="inlineStr">
+      <c r="B160" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -4978,7 +4985,7 @@
           <t>PO16569182</t>
         </is>
       </c>
-      <c r="B161" s="3" t="inlineStr">
+      <c r="B161" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5001,7 +5008,7 @@
           <t>PO16501867</t>
         </is>
       </c>
-      <c r="B162" s="3" t="inlineStr">
+      <c r="B162" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5024,7 +5031,7 @@
           <t>PO16390572</t>
         </is>
       </c>
-      <c r="B163" s="3" t="inlineStr">
+      <c r="B163" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5047,7 +5054,7 @@
           <t>PO16541834</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
+      <c r="B164" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5070,7 +5077,7 @@
           <t>PO14752925</t>
         </is>
       </c>
-      <c r="B165" s="3" t="inlineStr">
+      <c r="B165" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5093,7 +5100,7 @@
           <t>PO16435057</t>
         </is>
       </c>
-      <c r="B166" s="3" t="inlineStr">
+      <c r="B166" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5116,7 +5123,7 @@
           <t>PO16512210</t>
         </is>
       </c>
-      <c r="B167" s="3" t="inlineStr">
+      <c r="B167" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5139,7 +5146,7 @@
           <t>PO16386814</t>
         </is>
       </c>
-      <c r="B168" s="3" t="inlineStr">
+      <c r="B168" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5162,7 +5169,7 @@
           <t>PO16321781</t>
         </is>
       </c>
-      <c r="B169" s="3" t="inlineStr">
+      <c r="B169" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5185,7 +5192,7 @@
           <t>PO16255601</t>
         </is>
       </c>
-      <c r="B170" s="3" t="inlineStr">
+      <c r="B170" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5208,7 +5215,7 @@
           <t>PO16355659</t>
         </is>
       </c>
-      <c r="B171" s="3" t="inlineStr">
+      <c r="B171" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5231,7 +5238,7 @@
           <t>PO16489207</t>
         </is>
       </c>
-      <c r="B172" s="3" t="inlineStr">
+      <c r="B172" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5254,7 +5261,7 @@
           <t>PO15699499</t>
         </is>
       </c>
-      <c r="B173" s="3" t="inlineStr">
+      <c r="B173" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5277,7 +5284,7 @@
           <t>PO13622314</t>
         </is>
       </c>
-      <c r="B174" s="3" t="inlineStr">
+      <c r="B174" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5300,7 +5307,7 @@
           <t>PO15429046</t>
         </is>
       </c>
-      <c r="B175" s="3" t="inlineStr">
+      <c r="B175" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5323,7 +5330,7 @@
           <t>PO16394533</t>
         </is>
       </c>
-      <c r="B176" s="3" t="inlineStr">
+      <c r="B176" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5346,7 +5353,7 @@
           <t>PO16455498</t>
         </is>
       </c>
-      <c r="B177" s="3" t="inlineStr">
+      <c r="B177" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5369,7 +5376,7 @@
           <t>PO16326521</t>
         </is>
       </c>
-      <c r="B178" s="3" t="inlineStr">
+      <c r="B178" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5392,7 +5399,7 @@
           <t>PO15630092</t>
         </is>
       </c>
-      <c r="B179" s="3" t="inlineStr">
+      <c r="B179" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5415,7 +5422,7 @@
           <t>PO16433571</t>
         </is>
       </c>
-      <c r="B180" s="3" t="inlineStr">
+      <c r="B180" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5438,7 +5445,7 @@
           <t>PO16341901</t>
         </is>
       </c>
-      <c r="B181" s="3" t="inlineStr">
+      <c r="B181" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5461,7 +5468,7 @@
           <t>PO16064431</t>
         </is>
       </c>
-      <c r="B182" s="3" t="inlineStr">
+      <c r="B182" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5484,7 +5491,7 @@
           <t>PO14219870</t>
         </is>
       </c>
-      <c r="B183" s="3" t="inlineStr">
+      <c r="B183" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5507,7 +5514,7 @@
           <t>PO15630214</t>
         </is>
       </c>
-      <c r="B184" s="3" t="inlineStr">
+      <c r="B184" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5530,7 +5537,7 @@
           <t>PO15644153</t>
         </is>
       </c>
-      <c r="B185" s="3" t="inlineStr">
+      <c r="B185" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5553,7 +5560,7 @@
           <t>PO16256064</t>
         </is>
       </c>
-      <c r="B186" s="3" t="inlineStr">
+      <c r="B186" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5576,7 +5583,7 @@
           <t>PO15647942</t>
         </is>
       </c>
-      <c r="B187" s="3" t="inlineStr">
+      <c r="B187" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5599,7 +5606,7 @@
           <t>PO16322639</t>
         </is>
       </c>
-      <c r="B188" s="3" t="inlineStr">
+      <c r="B188" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5622,7 +5629,7 @@
           <t>PO16329589</t>
         </is>
       </c>
-      <c r="B189" s="3" t="inlineStr">
+      <c r="B189" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5645,7 +5652,7 @@
           <t>PO16184045</t>
         </is>
       </c>
-      <c r="B190" s="3" t="inlineStr">
+      <c r="B190" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5668,7 +5675,7 @@
           <t>PO16495607</t>
         </is>
       </c>
-      <c r="B191" s="3" t="inlineStr">
+      <c r="B191" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5691,7 +5698,7 @@
           <t>PO16438043</t>
         </is>
       </c>
-      <c r="B192" s="3" t="inlineStr">
+      <c r="B192" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5714,7 +5721,7 @@
           <t>PO15014528</t>
         </is>
       </c>
-      <c r="B193" s="3" t="inlineStr">
+      <c r="B193" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5737,7 +5744,7 @@
           <t>PO16299456</t>
         </is>
       </c>
-      <c r="B194" s="3" t="inlineStr">
+      <c r="B194" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5760,7 +5767,7 @@
           <t>PO16433499</t>
         </is>
       </c>
-      <c r="B195" s="3" t="inlineStr">
+      <c r="B195" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5783,7 +5790,7 @@
           <t>PO16441737</t>
         </is>
       </c>
-      <c r="B196" s="3" t="inlineStr">
+      <c r="B196" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5806,7 +5813,7 @@
           <t>PO15694769</t>
         </is>
       </c>
-      <c r="B197" s="3" t="inlineStr">
+      <c r="B197" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5829,7 +5836,7 @@
           <t>PO15694772</t>
         </is>
       </c>
-      <c r="B198" s="3" t="inlineStr">
+      <c r="B198" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5852,7 +5859,7 @@
           <t>PO16496851</t>
         </is>
       </c>
-      <c r="B199" s="3" t="inlineStr">
+      <c r="B199" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5875,7 +5882,7 @@
           <t>PO13653137</t>
         </is>
       </c>
-      <c r="B200" s="3" t="inlineStr">
+      <c r="B200" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5898,7 +5905,7 @@
           <t>PO16389062</t>
         </is>
       </c>
-      <c r="B201" s="3" t="inlineStr">
+      <c r="B201" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5921,7 +5928,7 @@
           <t>PO15695018</t>
         </is>
       </c>
-      <c r="B202" s="3" t="inlineStr">
+      <c r="B202" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5944,7 +5951,7 @@
           <t>PO16152224</t>
         </is>
       </c>
-      <c r="B203" s="3" t="inlineStr">
+      <c r="B203" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5967,7 +5974,7 @@
           <t>PO16511466</t>
         </is>
       </c>
-      <c r="B204" s="3" t="inlineStr">
+      <c r="B204" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -5990,7 +5997,7 @@
           <t>PO16191221</t>
         </is>
       </c>
-      <c r="B205" s="3" t="inlineStr">
+      <c r="B205" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6013,7 +6020,7 @@
           <t>PO14752926</t>
         </is>
       </c>
-      <c r="B206" s="3" t="inlineStr">
+      <c r="B206" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6036,7 +6043,7 @@
           <t>PO15628885</t>
         </is>
       </c>
-      <c r="B207" s="3" t="inlineStr">
+      <c r="B207" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6059,7 +6066,7 @@
           <t>PO16314188</t>
         </is>
       </c>
-      <c r="B208" s="3" t="inlineStr">
+      <c r="B208" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6082,7 +6089,7 @@
           <t>PO14607065</t>
         </is>
       </c>
-      <c r="B209" s="3" t="inlineStr">
+      <c r="B209" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6105,7 +6112,7 @@
           <t>PO16064432</t>
         </is>
       </c>
-      <c r="B210" s="3" t="inlineStr">
+      <c r="B210" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6128,7 +6135,7 @@
           <t>PO16340514</t>
         </is>
       </c>
-      <c r="B211" s="3" t="inlineStr">
+      <c r="B211" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6151,7 +6158,7 @@
           <t>PO16006846</t>
         </is>
       </c>
-      <c r="B212" s="3" t="inlineStr">
+      <c r="B212" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6174,7 +6181,7 @@
           <t>PO15630301</t>
         </is>
       </c>
-      <c r="B213" s="3" t="inlineStr">
+      <c r="B213" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6197,7 +6204,7 @@
           <t>PO16243291</t>
         </is>
       </c>
-      <c r="B214" s="3" t="inlineStr">
+      <c r="B214" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6220,7 +6227,7 @@
           <t>PO16450524</t>
         </is>
       </c>
-      <c r="B215" s="3" t="inlineStr">
+      <c r="B215" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6243,7 +6250,7 @@
           <t>PO16518287</t>
         </is>
       </c>
-      <c r="B216" s="3" t="inlineStr">
+      <c r="B216" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6266,7 +6273,7 @@
           <t>PO16501626</t>
         </is>
       </c>
-      <c r="B217" s="3" t="inlineStr">
+      <c r="B217" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6289,7 +6296,7 @@
           <t>PO14065853</t>
         </is>
       </c>
-      <c r="B218" s="3" t="inlineStr">
+      <c r="B218" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6312,7 +6319,7 @@
           <t>PO15694770</t>
         </is>
       </c>
-      <c r="B219" s="3" t="inlineStr">
+      <c r="B219" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6335,7 +6342,7 @@
           <t>PO16501625</t>
         </is>
       </c>
-      <c r="B220" s="3" t="inlineStr">
+      <c r="B220" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6358,7 +6365,7 @@
           <t>PO16396709</t>
         </is>
       </c>
-      <c r="B221" s="3" t="inlineStr">
+      <c r="B221" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6381,7 +6388,7 @@
           <t>PO16404433</t>
         </is>
       </c>
-      <c r="B222" s="3" t="inlineStr">
+      <c r="B222" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6404,7 +6411,7 @@
           <t>PO16356881</t>
         </is>
       </c>
-      <c r="B223" s="3" t="inlineStr">
+      <c r="B223" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6427,7 +6434,7 @@
           <t>PO15694761</t>
         </is>
       </c>
-      <c r="B224" s="3" t="inlineStr">
+      <c r="B224" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6450,7 +6457,7 @@
           <t>PO15613054</t>
         </is>
       </c>
-      <c r="B225" s="3" t="inlineStr">
+      <c r="B225" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6473,7 +6480,7 @@
           <t>PO15630315</t>
         </is>
       </c>
-      <c r="B226" s="3" t="inlineStr">
+      <c r="B226" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6496,7 +6503,7 @@
           <t>PO15694762</t>
         </is>
       </c>
-      <c r="B227" s="3" t="inlineStr">
+      <c r="B227" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6519,7 +6526,7 @@
           <t>PO16370804</t>
         </is>
       </c>
-      <c r="B228" s="3" t="inlineStr">
+      <c r="B228" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6542,7 +6549,7 @@
           <t>PO16145734</t>
         </is>
       </c>
-      <c r="B229" s="3" t="inlineStr">
+      <c r="B229" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6565,7 +6572,7 @@
           <t>PO16361280</t>
         </is>
       </c>
-      <c r="B230" s="3" t="inlineStr">
+      <c r="B230" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6588,7 +6595,7 @@
           <t>PO15699771</t>
         </is>
       </c>
-      <c r="B231" s="3" t="inlineStr">
+      <c r="B231" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6611,7 +6618,7 @@
           <t>PO16362352</t>
         </is>
       </c>
-      <c r="B232" s="3" t="inlineStr">
+      <c r="B232" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6634,7 +6641,7 @@
           <t>PO16530239</t>
         </is>
       </c>
-      <c r="B233" s="3" t="inlineStr">
+      <c r="B233" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6657,7 +6664,7 @@
           <t>PO16051893</t>
         </is>
       </c>
-      <c r="B234" s="3" t="inlineStr">
+      <c r="B234" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6680,7 +6687,7 @@
           <t>PO16330375</t>
         </is>
       </c>
-      <c r="B235" s="3" t="inlineStr">
+      <c r="B235" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6703,7 +6710,7 @@
           <t>PO15241466</t>
         </is>
       </c>
-      <c r="B236" s="3" t="inlineStr">
+      <c r="B236" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6726,7 +6733,7 @@
           <t>PO16442571</t>
         </is>
       </c>
-      <c r="B237" s="3" t="inlineStr">
+      <c r="B237" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6749,7 +6756,7 @@
           <t>PO16157599</t>
         </is>
       </c>
-      <c r="B238" s="3" t="inlineStr">
+      <c r="B238" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6772,7 +6779,7 @@
           <t>PO14738382</t>
         </is>
       </c>
-      <c r="B239" s="3" t="inlineStr">
+      <c r="B239" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6795,7 +6802,7 @@
           <t>PO14760883</t>
         </is>
       </c>
-      <c r="B240" s="3" t="inlineStr">
+      <c r="B240" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6818,7 +6825,7 @@
           <t>PO14719278</t>
         </is>
       </c>
-      <c r="B241" s="3" t="inlineStr">
+      <c r="B241" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6841,7 +6848,7 @@
           <t>PO14760850</t>
         </is>
       </c>
-      <c r="B242" s="3" t="inlineStr">
+      <c r="B242" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6864,7 +6871,7 @@
           <t>PO14719338</t>
         </is>
       </c>
-      <c r="B243" s="3" t="inlineStr">
+      <c r="B243" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6887,7 +6894,7 @@
           <t>PO16359448</t>
         </is>
       </c>
-      <c r="B244" s="3" t="inlineStr">
+      <c r="B244" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6910,7 +6917,7 @@
           <t>PO16547176</t>
         </is>
       </c>
-      <c r="B245" s="3" t="inlineStr">
+      <c r="B245" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6933,7 +6940,7 @@
           <t>PO14010216</t>
         </is>
       </c>
-      <c r="B246" s="3" t="inlineStr">
+      <c r="B246" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6956,7 +6963,7 @@
           <t>PO14010221</t>
         </is>
       </c>
-      <c r="B247" s="3" t="inlineStr">
+      <c r="B247" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -6979,7 +6986,7 @@
           <t>PO16323002</t>
         </is>
       </c>
-      <c r="B248" s="3" t="inlineStr">
+      <c r="B248" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7002,7 +7009,7 @@
           <t>PO16315115</t>
         </is>
       </c>
-      <c r="B249" s="3" t="inlineStr">
+      <c r="B249" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7025,7 +7032,7 @@
           <t>PO16488717</t>
         </is>
       </c>
-      <c r="B250" s="3" t="inlineStr">
+      <c r="B250" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7048,7 +7055,7 @@
           <t>PO16522171</t>
         </is>
       </c>
-      <c r="B251" s="3" t="inlineStr">
+      <c r="B251" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7071,7 +7078,7 @@
           <t>PO16485947</t>
         </is>
       </c>
-      <c r="B252" s="3" t="inlineStr">
+      <c r="B252" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7094,7 +7101,7 @@
           <t>PO15874912</t>
         </is>
       </c>
-      <c r="B253" s="3" t="inlineStr">
+      <c r="B253" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7117,7 +7124,7 @@
           <t>PO13064901</t>
         </is>
       </c>
-      <c r="B254" s="3" t="inlineStr">
+      <c r="B254" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7140,7 +7147,7 @@
           <t>PO15614578</t>
         </is>
       </c>
-      <c r="B255" s="3" t="inlineStr">
+      <c r="B255" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7163,7 +7170,7 @@
           <t>PO16224336</t>
         </is>
       </c>
-      <c r="B256" s="3" t="inlineStr">
+      <c r="B256" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7186,7 +7193,7 @@
           <t>PO16207339</t>
         </is>
       </c>
-      <c r="B257" s="3" t="inlineStr">
+      <c r="B257" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7209,7 +7216,7 @@
           <t>PO14010218</t>
         </is>
       </c>
-      <c r="B258" s="3" t="inlineStr">
+      <c r="B258" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7232,7 +7239,7 @@
           <t>PO16202587</t>
         </is>
       </c>
-      <c r="B259" s="3" t="inlineStr">
+      <c r="B259" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7255,7 +7262,7 @@
           <t>PO16211797</t>
         </is>
       </c>
-      <c r="B260" s="3" t="inlineStr">
+      <c r="B260" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7278,7 +7285,7 @@
           <t>PO15220371</t>
         </is>
       </c>
-      <c r="B261" s="3" t="inlineStr">
+      <c r="B261" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7301,7 +7308,7 @@
           <t>PO16271627</t>
         </is>
       </c>
-      <c r="B262" s="3" t="inlineStr">
+      <c r="B262" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7324,7 +7331,7 @@
           <t>PO16264130</t>
         </is>
       </c>
-      <c r="B263" s="3" t="inlineStr">
+      <c r="B263" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7347,7 +7354,7 @@
           <t>PO14008887</t>
         </is>
       </c>
-      <c r="B264" s="3" t="inlineStr">
+      <c r="B264" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7370,7 +7377,7 @@
           <t>PO14958078</t>
         </is>
       </c>
-      <c r="B265" s="3" t="inlineStr">
+      <c r="B265" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7393,7 +7400,7 @@
           <t>PO13406596</t>
         </is>
       </c>
-      <c r="B266" s="3" t="inlineStr">
+      <c r="B266" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7416,7 +7423,7 @@
           <t>PO15220377</t>
         </is>
       </c>
-      <c r="B267" s="3" t="inlineStr">
+      <c r="B267" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
@@ -7439,7 +7446,7 @@
           <t>PO13247181</t>
         </is>
       </c>
-      <c r="B268" s="3" t="inlineStr">
+      <c r="B268" s="4" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>

</xml_diff>